<commit_message>
hapus tabel program academik
</commit_message>
<xml_diff>
--- a/scripts/output/dosen_universitas_ngudi_waluyo.xlsx
+++ b/scripts/output/dosen_universitas_ngudi_waluyo.xlsx
@@ -1779,22 +1779,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ANA PUJI ASTUTI</t>
+          <t>AGITYA RESTI ERWIYANI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>6146672</t>
+          <t>6082202</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Keperawatan (D3)</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 12</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1805,44 +1805,44 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>471</t>
+          <t>566</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>70</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>115</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6146672</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082202</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AGITYA RESTI ERWIYANI</t>
+          <t>ANA PUJI ASTUTI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>6082202</t>
+          <t>6146672</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Keperawatan (D3)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 12</t>
+          <t>Scopus H-Index : 0GS H-Index : 7</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1853,22 +1853,22 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>566</t>
+          <t>471</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>170</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>170</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082202</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6146672</t>
         </is>
       </c>
     </row>
@@ -1971,22 +1971,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PUJI LESTARI</t>
+          <t>IKA NILAWATI</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>6093197</t>
+          <t>6785923</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Keperawatan (S1)</t>
+          <t>Ilmu Keolahragaan (S1)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 10</t>
+          <t>Scopus H-Index : 0GS H-Index : 4</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -1997,44 +1997,44 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>303</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>150</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>195</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6093197</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6785923</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>IKA NILAWATI</t>
+          <t>PUJI LESTARI</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>6785923</t>
+          <t>6093197</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ilmu Keolahragaan (S1)</t>
+          <t>Keperawatan (S1)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 4</t>
+          <t>Scopus H-Index : 0GS H-Index : 10</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -2045,22 +2045,22 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>530</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>130</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6785923</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6093197</t>
         </is>
       </c>
     </row>
@@ -3699,22 +3699,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>RATIH LAILY NURJANAH</t>
+          <t>HERI SUGIARTO</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>6199137</t>
+          <t>5985236</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Sastra Inggris (S1)</t>
+          <t>Kesehatan Masyarakat (S1)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 2GS H-Index : 5</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -3725,44 +3725,44 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>372</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>55</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>85</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6199137</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/5985236</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>HERI SUGIARTO</t>
+          <t>RATIH LAILY NURJANAH</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>5985236</t>
+          <t>6199137</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Kesehatan Masyarakat (S1)</t>
+          <t>Sastra Inggris (S1)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 2GS H-Index : 5</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -3773,22 +3773,22 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>372</t>
+          <t>459</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/5985236</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6199137</t>
         </is>
       </c>
     </row>
@@ -5715,17 +5715,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ARDA RADITYA TANTRA</t>
+          <t>AR-RAHIIM INNASH</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>6832181</t>
+          <t>6895455</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Akuntansi Perpajakan (D4)</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -5741,39 +5741,39 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>113</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>45</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6832181</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895455</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ARDA RADITYA TANTRA</t>
+          <t>AR-RAHIIM INNASH</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>6832181</t>
+          <t>6895455</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Akuntansi Perpajakan (D4)</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -5789,44 +5789,44 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>113</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>45</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6832181</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895455</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>PUJI AFIATNA</t>
+          <t>GUNTUR RATIH PRESTIFA HERDINATA</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>6198595</t>
+          <t>6828552</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Gizi (S1)</t>
+          <t>Ilmu Keolahragaan (S1)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 2GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 3</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
@@ -5837,44 +5837,44 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>198</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>120</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198595</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828552</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>GUNTUR RATIH PRESTIFA HERDINATA</t>
+          <t>PUJI AFIATNA</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>6828552</t>
+          <t>6198595</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Ilmu Keolahragaan (S1)</t>
+          <t>Gizi (S1)</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 3</t>
+          <t>Scopus H-Index : 2GS H-Index : 7</t>
         </is>
       </c>
       <c r="E114" t="inlineStr"/>
@@ -5885,22 +5885,22 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>194</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>30</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828552</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198595</t>
         </is>
       </c>
     </row>
@@ -8019,22 +8019,22 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>FITRIA PRIMI ASTUTI</t>
+          <t>INDAH KURNIAWATI</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>6082432</t>
+          <t>6910777</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E159" t="inlineStr"/>
@@ -8045,7 +8045,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>174</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -8060,19 +8060,19 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082432</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910777</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ANDI PRADANA</t>
+          <t>SITI KHOIRIYAH</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>6910783</t>
+          <t>6910724</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -8082,7 +8082,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 1</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
@@ -8093,7 +8093,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -8108,29 +8108,29 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910783</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910724</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>INDAH KURNIAWATI</t>
+          <t>FITRIA PRIMI ASTUTI</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>6910777</t>
+          <t>6082432</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 0GS H-Index : 7</t>
         </is>
       </c>
       <c r="E161" t="inlineStr"/>
@@ -8141,7 +8141,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>174</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
@@ -8156,19 +8156,19 @@
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910777</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082432</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>SITI KHOIRIYAH</t>
+          <t>INDAH KURNIAWATI</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>6910724</t>
+          <t>6910777</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -8204,24 +8204,24 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910724</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910777</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>DWI WISNU KURNIAWAN</t>
+          <t>DWI RETNA SUSILOWATI</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>6967441</t>
+          <t>6895451</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Ilmu Hukum (S1)</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -8237,7 +8237,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -8252,19 +8252,19 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967441</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895451</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>FIKRI ARIYAD</t>
+          <t>ADI PURWANTO</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>6837372</t>
+          <t>6198866</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -8285,44 +8285,44 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr">
+      <c r="I164" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="I164" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6837372</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198866</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>MUFTI AGUNG WIBOWO</t>
+          <t>DWI WISNU KURNIAWAN</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>6871253</t>
+          <t>6967441</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Bisnis Digital (S1)</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 1GS H-Index : 0</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
@@ -8333,7 +8333,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -8343,29 +8343,29 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6871253</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967441</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>DWI RETNA SUSILOWATI</t>
+          <t>FIKRI ARIYAD</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>6895451</t>
+          <t>6837372</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -8396,29 +8396,29 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895451</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6837372</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>ADI PURWANTO</t>
+          <t>MUFTI AGUNG WIBOWO</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>6198866</t>
+          <t>6871253</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Bisnis Digital (S1)</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 1GS H-Index : 0</t>
         </is>
       </c>
       <c r="E167" t="inlineStr"/>
@@ -8429,7 +8429,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>114</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
@@ -8439,12 +8439,12 @@
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198866</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6871253</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
perfix pivot addjust dosen tabel
</commit_message>
<xml_diff>
--- a/scripts/output/dosen_universitas_ngudi_waluyo.xlsx
+++ b/scripts/output/dosen_universitas_ngudi_waluyo.xlsx
@@ -915,17 +915,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SITI HARYANI</t>
+          <t>UMI ANIROH</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>6136655</t>
+          <t>6198559</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Keperawatan (D3)</t>
+          <t>Profesi Ners (Profesi)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -941,22 +941,22 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>681</t>
+          <t>816</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>230</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>205</t>
+          <t>460</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6136655</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198559</t>
         </is>
       </c>
     </row>
@@ -978,18 +978,18 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 9</t>
+          <t>Scopus H-Index : 0GS H-Index : 10</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>332</t>
+          <t>337</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>796</t>
+          <t>816</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1779,22 +1779,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AGITYA RESTI ERWIYANI</t>
+          <t>ANA PUJI ASTUTI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>6082202</t>
+          <t>6146672</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Keperawatan (D3)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 12</t>
+          <t>Scopus H-Index : 0GS H-Index : 7</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1805,44 +1805,44 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>566</t>
+          <t>471</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>170</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>170</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082202</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6146672</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ANA PUJI ASTUTI</t>
+          <t>AGITYA RESTI ERWIYANI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>6146672</t>
+          <t>6082202</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Keperawatan (D3)</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 12</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1853,22 +1853,22 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>471</t>
+          <t>566</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>70</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>115</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6146672</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6082202</t>
         </is>
       </c>
     </row>
@@ -2643,113 +2643,113 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>EKO NUR HERMANSYAH</t>
+          <t>MELATI APRILLIANA RAMADHANI</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>6904295</t>
+          <t>6755940</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Bisnis Digital (S1)</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 4</t>
+          <t>Scopus H-Index : 0GS H-Index : 7</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>202</t>
+          <t>201</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>275</t>
+          <t>376</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>150</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>200</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6904295</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6755940</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>MELATI APRILLIANA RAMADHANI</t>
+          <t>WULANSARI</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>6755940</t>
+          <t>6150389</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Keperawatan (D3)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 6</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>196</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>376</t>
+          <t>414</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>90</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>175</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6755940</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6150389</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>WULANSARI</t>
+          <t>RISMA ALIVIANI PUTRI</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>6150389</t>
+          <t>6083924</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Keperawatan (D3)</t>
+          <t>Kebidanan (S1)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2760,171 +2760,171 @@
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>195</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>414</t>
+          <t>518</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>175</t>
+          <t>95</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6150389</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6083924</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>RISMA ALIVIANI PUTRI</t>
+          <t>SITI MUTMAINAH</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>6083924</t>
+          <t>6927670</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Kebidanan (S1)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 6</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>192</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>518</t>
+          <t>264</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6083924</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6927670</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SITI MUTMAINAH</t>
+          <t>SIGIT AMBAR WIDYAWATI</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>6927670</t>
+          <t>6116540</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Kesehatan Masyarakat (S1)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 1GS H-Index : 8</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t>192</t>
+          <t>189</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>264</t>
+          <t>490</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>70</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>115</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6927670</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6116540</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SIGIT AMBAR WIDYAWATI</t>
+          <t>EKO NUR HERMANSYAH</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>6116540</t>
+          <t>6904295</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Kesehatan Masyarakat (S1)</t>
+          <t>Bisnis Digital (S1)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 1GS H-Index : 8</t>
+          <t>Scopus H-Index : 0GS H-Index : 4</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>183</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>490</t>
+          <t>260</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>95</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>105</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6116540</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6904295</t>
         </is>
       </c>
     </row>
@@ -3171,22 +3171,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ISFAIZAH</t>
+          <t>FIKTINA VIFRI ISMIRIYAM</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>6085376</t>
+          <t>6138998</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Kebidanan (S1)</t>
+          <t>Keperawatan (D3)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 6</t>
+          <t>Scopus H-Index : 0GS H-Index : 5</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -3197,44 +3197,44 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>391</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>85</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>175</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6085376</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6138998</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>FIKTINA VIFRI ISMIRIYAM</t>
+          <t>ISFAIZAH</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>6138998</t>
+          <t>6085376</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Keperawatan (D3)</t>
+          <t>Kebidanan (S1)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 5</t>
+          <t>Scopus H-Index : 0GS H-Index : 6</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -3245,22 +3245,22 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>391</t>
+          <t>510</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>0</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>175</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6138998</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6085376</t>
         </is>
       </c>
     </row>
@@ -5357,7 +5357,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>289</t>
+          <t>290</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -5715,17 +5715,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>AR-RAHIIM INNASH</t>
+          <t>ARDA RADITYA TANTRA</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>6895455</t>
+          <t>6832181</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Ilmu Hukum (S1)</t>
+          <t>Akuntansi Perpajakan (D4)</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -5741,39 +5741,39 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>138</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895455</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6832181</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>AR-RAHIIM INNASH</t>
+          <t>ARDA RADITYA TANTRA</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>6895455</t>
+          <t>6832181</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Ilmu Hukum (S1)</t>
+          <t>Akuntansi Perpajakan (D4)</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -5789,44 +5789,44 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>138</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895455</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6832181</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>GUNTUR RATIH PRESTIFA HERDINATA</t>
+          <t>PUJI AFIATNA</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>6828552</t>
+          <t>6198595</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Ilmu Keolahragaan (S1)</t>
+          <t>Gizi (S1)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 3</t>
+          <t>Scopus H-Index : 2GS H-Index : 7</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
@@ -5837,44 +5837,44 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>194</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>30</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828552</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198595</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>PUJI AFIATNA</t>
+          <t>GUNTUR RATIH PRESTIFA HERDINATA</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>6198595</t>
+          <t>6828552</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Gizi (S1)</t>
+          <t>Ilmu Keolahragaan (S1)</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 2GS H-Index : 7</t>
+          <t>Scopus H-Index : 0GS H-Index : 3</t>
         </is>
       </c>
       <c r="E114" t="inlineStr"/>
@@ -5885,22 +5885,22 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>198</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>40</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>120</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198595</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6828552</t>
         </is>
       </c>
     </row>
@@ -7923,22 +7923,22 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>SUKARNO</t>
+          <t>TUSI WIRAHAYU PERTIWI</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>6198543</t>
+          <t>6967446</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Keperawatan (S1)</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 14</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E157" t="inlineStr"/>
@@ -7949,7 +7949,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -7964,29 +7964,29 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198543</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967446</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>TUSI WIRAHAYU PERTIWI</t>
+          <t>SUKARNO</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>6967446</t>
+          <t>6198543</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Ilmu Hukum (S1)</t>
+          <t>Keperawatan (S1)</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 0GS H-Index : 14</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
@@ -7997,7 +7997,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>356</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -8012,19 +8012,19 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967446</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198543</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>INDAH KURNIAWATI</t>
+          <t>SITI KHOIRIYAH</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>6910777</t>
+          <t>6910724</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -8060,19 +8060,19 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910777</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910724</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>SITI KHOIRIYAH</t>
+          <t>ANDI PRADANA</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>6910724</t>
+          <t>6910783</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -8082,7 +8082,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 0GS H-Index : 1</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
@@ -8093,7 +8093,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -8108,7 +8108,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910724</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910783</t>
         </is>
       </c>
     </row>
@@ -8163,12 +8163,12 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>INDAH KURNIAWATI</t>
+          <t>SITI KHOIRIYAH</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>6910777</t>
+          <t>6910724</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -8204,24 +8204,24 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910777</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6910724</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>DWI RETNA SUSILOWATI</t>
+          <t>DWI WISNU KURNIAWAN</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>6895451</t>
+          <t>6967441</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Farmasi (S1)</t>
+          <t>Ilmu Hukum (S1)</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -8237,34 +8237,34 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr">
+      <c r="I163" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="I163" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895451</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967441</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>ADI PURWANTO</t>
+          <t>FIKRI ARIYAD</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>6198866</t>
+          <t>6837372</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -8285,7 +8285,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
@@ -8300,29 +8300,29 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198866</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6837372</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>DWI WISNU KURNIAWAN</t>
+          <t>MUFTI AGUNG WIBOWO</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>6967441</t>
+          <t>6871253</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Ilmu Hukum (S1)</t>
+          <t>Bisnis Digital (S1)</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 0GS H-Index : 0</t>
+          <t>Scopus H-Index : 1GS H-Index : 0</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
@@ -8333,7 +8333,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>114</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -8343,29 +8343,29 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6967441</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6871253</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>FIKRI ARIYAD</t>
+          <t>DWI RETNA SUSILOWATI</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>6837372</t>
+          <t>6895451</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Farmasi (S1)</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -8396,29 +8396,29 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6837372</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6895451</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>MUFTI AGUNG WIBOWO</t>
+          <t>ADI PURWANTO</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>6871253</t>
+          <t>6198866</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Bisnis Digital (S1)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Scopus H-Index : 1GS H-Index : 0</t>
+          <t>Scopus H-Index : 0GS H-Index : 0</t>
         </is>
       </c>
       <c r="E167" t="inlineStr"/>
@@ -8429,7 +8429,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
@@ -8439,12 +8439,12 @@
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6871253</t>
+          <t>https://sinta.kemdiktisaintek.go.id/authors/profile/6198866</t>
         </is>
       </c>
     </row>

</xml_diff>